<commit_message>
feat(onboarding): advance validated partner forms
</commit_message>
<xml_diff>
--- a/outputs/partner-form-template/VPN_MVT_M-MOLA_PUSHUSSD_PartnerName_074613_UPDATED.xlsx
+++ b/outputs/partner-form-template/VPN_MVT_M-MOLA_PUSHUSSD_PartnerName_074613_UPDATED.xlsx
@@ -455,7 +455,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z42"/>
+  <dimension ref="A1:Z43"/>
   <cols>
     <col min="1" max="1" width="28.5" customWidth="1"/>
     <col min="2" max="2" width="30.5" customWidth="1"/>
@@ -1109,7 +1109,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Technical Contact Details</v>
+        <v>Group Link</v>
       </c>
       <c r="B9" t="str">
         <v/>
@@ -1189,7 +1189,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Primary</v>
+        <v>Technical Contact Details</v>
       </c>
       <c r="B10" t="str">
         <v/>
@@ -1269,13 +1269,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Name</v>
+        <v>Primary</v>
       </c>
       <c r="B11" t="str">
-        <v>Isodoro Onório</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>Xefino José</v>
+        <v/>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -1349,13 +1349,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Email Address</v>
+        <v>Name</v>
       </c>
       <c r="B12" t="str">
-        <v>ernestoioj@movitel.co.mz</v>
+        <v>Isodoro Onório</v>
       </c>
       <c r="C12" t="str">
-        <v>ondetem.dev@gmail.com</v>
+        <v>Xefino José</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -1429,13 +1429,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Desk Phone</v>
+        <v>Email Address</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>ernestoioj@movitel.co.mz</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>ondetem.dev@gmail.com</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -1509,13 +1509,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Cell Phone</v>
+        <v>Desk Phone</v>
       </c>
       <c r="B14" t="str">
-        <v>+258872315305</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>+258 876337381</v>
+        <v/>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -1589,13 +1589,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Skype</v>
+        <v>Cell Phone</v>
       </c>
       <c r="B15" t="str">
-        <v>Isidoro Onório</v>
+        <v>+258872315305</v>
       </c>
       <c r="C15" t="str">
-        <v>Xefino José</v>
+        <v>+258 876337381</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Secondary</v>
+        <v>Skype</v>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v>Isidoro Onório</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>Xefino José</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -1749,13 +1749,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Name</v>
+        <v>Secondary</v>
       </c>
       <c r="B17" t="str">
-        <v>Donaldo Polane</v>
+        <v/>
       </c>
       <c r="C17" t="str">
-        <v>Dino Zeca Iassido</v>
+        <v/>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -1829,13 +1829,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Email Address</v>
+        <v>Name</v>
       </c>
       <c r="B18" t="str">
-        <v>Donaldo.polane@movitel.co.mz</v>
+        <v>Donaldo Polane</v>
       </c>
       <c r="C18" t="str">
-        <v>zecadino674@gmail.com</v>
+        <v>Dino Zeca Iassido</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -1909,13 +1909,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Desk Phone</v>
+        <v>Email Address</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>Donaldo.polane@movitel.co.mz</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>zecadino674@gmail.com</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -1989,13 +1989,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Cell Phone</v>
+        <v>Desk Phone</v>
       </c>
       <c r="B20" t="str">
-        <v>+258 864221318</v>
-      </c>
-      <c r="C20">
-        <v>258878864136</v>
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -2069,13 +2069,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Skype</v>
+        <v>Cell Phone</v>
       </c>
       <c r="B21" t="str">
-        <v>Donaldo Polane</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Dino Zeca Iassido</v>
+        <v>+258 864221318</v>
+      </c>
+      <c r="C21">
+        <v>258878864136</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -2149,13 +2149,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>VPN Technical Details</v>
+        <v>Skype</v>
       </c>
       <c r="B22" t="str">
-        <v>Movitel  Preferred Config</v>
+        <v>Donaldo Polane</v>
       </c>
       <c r="C22" t="str">
-        <v>Partner name  Preferred Config</v>
+        <v>Dino Zeca Iassido</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>VPN Peer Address</v>
+        <v>VPN Technical Details</v>
       </c>
       <c r="B23" t="str">
-        <v>197.218.1.250</v>
+        <v>Movitel  Preferred Config</v>
       </c>
       <c r="C23" t="str">
-        <v xml:space="preserve"> 34.1.210.78</v>
+        <v>Partner name  Preferred Config</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -2309,13 +2309,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">VPN Device </v>
+        <v>VPN Peer Address</v>
       </c>
       <c r="B24" t="str">
-        <v>Fortigate</v>
+        <v>197.218.1.250</v>
       </c>
       <c r="C24" t="str">
-        <v>Linux strongSwan</v>
+        <v xml:space="preserve"> 34.1.210.78</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -2389,13 +2389,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>VPN Device Version</v>
+        <v xml:space="preserve">VPN Device </v>
       </c>
       <c r="B25" t="str">
-        <v>1200D</v>
+        <v>Fortigate</v>
       </c>
       <c r="C25" t="str">
-        <v>5.9.8</v>
+        <v>Linux strongSwan</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -2469,89 +2469,169 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>VPN Device Version</v>
+      </c>
+      <c r="B26" t="str">
+        <v>1200D</v>
+      </c>
+      <c r="C26" t="str">
+        <v>5.9.8</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+      <c r="Z26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>VPN Device Location</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B27" t="str">
         <v>Maputo</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C27" t="str">
         <v>africa-south1-b</v>
       </c>
-      <c r="D26" t="str">
-        <v/>
-      </c>
-      <c r="E26" t="str">
-        <v/>
-      </c>
-      <c r="F26" t="str">
-        <v/>
-      </c>
-      <c r="G26" t="str">
-        <v/>
-      </c>
-      <c r="H26" t="str">
-        <v/>
-      </c>
-      <c r="I26" t="str">
-        <v/>
-      </c>
-      <c r="J26" t="str">
-        <v/>
-      </c>
-      <c r="K26" t="str">
-        <v/>
-      </c>
-      <c r="L26" t="str">
-        <v/>
-      </c>
-      <c r="M26" t="str">
-        <v/>
-      </c>
-      <c r="N26" t="str">
-        <v/>
-      </c>
-      <c r="O26" t="str">
-        <v/>
-      </c>
-      <c r="P26" t="str">
-        <v/>
-      </c>
-      <c r="Q26" t="str">
-        <v/>
-      </c>
-      <c r="R26" t="str">
-        <v/>
-      </c>
-      <c r="S26" t="str">
-        <v/>
-      </c>
-      <c r="T26" t="str">
-        <v/>
-      </c>
-      <c r="U26" t="str">
-        <v/>
-      </c>
-      <c r="V26" t="str">
-        <v/>
-      </c>
-      <c r="W26" t="str">
-        <v/>
-      </c>
-      <c r="X26" t="str">
-        <v/>
-      </c>
-      <c r="Y26" t="str">
-        <v/>
-      </c>
-      <c r="Z26" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str">
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
+      </c>
+      <c r="Z27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
         <v xml:space="preserve">Encryption domain </v>
       </c>
-      <c r="B27" t="str" xml:space="preserve">
+      <c r="B28" t="str" xml:space="preserve">
         <v xml:space="preserve"> 10.229.16.29
  10.229.16.30
  10.229.42.197
@@ -2559,88 +2639,8 @@
 10.229.41.49
 </v>
       </c>
-      <c r="C27" t="str">
+      <c r="C28" t="str">
         <v>10.218.0.2/32</v>
-      </c>
-      <c r="D27" t="str">
-        <v/>
-      </c>
-      <c r="E27" t="str">
-        <v/>
-      </c>
-      <c r="F27" t="str">
-        <v/>
-      </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
-      <c r="H27" t="str">
-        <v/>
-      </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
-      <c r="J27" t="str">
-        <v/>
-      </c>
-      <c r="K27" t="str">
-        <v/>
-      </c>
-      <c r="L27" t="str">
-        <v/>
-      </c>
-      <c r="M27" t="str">
-        <v/>
-      </c>
-      <c r="N27" t="str">
-        <v/>
-      </c>
-      <c r="O27" t="str">
-        <v/>
-      </c>
-      <c r="P27" t="str">
-        <v/>
-      </c>
-      <c r="Q27" t="str">
-        <v/>
-      </c>
-      <c r="R27" t="str">
-        <v/>
-      </c>
-      <c r="S27" t="str">
-        <v/>
-      </c>
-      <c r="T27" t="str">
-        <v/>
-      </c>
-      <c r="U27" t="str">
-        <v/>
-      </c>
-      <c r="V27" t="str">
-        <v/>
-      </c>
-      <c r="W27" t="str">
-        <v/>
-      </c>
-      <c r="X27" t="str">
-        <v/>
-      </c>
-      <c r="Y27" t="str">
-        <v/>
-      </c>
-      <c r="Z27" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>IKE Phase 1 Parameters</v>
-      </c>
-      <c r="B28" t="str">
-        <v/>
-      </c>
-      <c r="C28" t="str">
-        <v/>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -2714,10 +2714,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Authentication Method</v>
+        <v>IKE Phase 1 Parameters</v>
       </c>
       <c r="B29" t="str">
-        <v>Pre-share Key (PSK)</v>
+        <v/>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -2794,13 +2794,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Encryption Scheme</v>
+        <v>Authentication Method</v>
       </c>
       <c r="B30" t="str">
-        <v>IKEv2</v>
+        <v>Pre-share Key (PSK)</v>
       </c>
       <c r="C30" t="str">
-        <v>IKEv2</v>
+        <v/>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -2874,13 +2874,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Diffie-Hellman Group</v>
+        <v>Encryption Scheme</v>
       </c>
       <c r="B31" t="str">
-        <v>Group 14</v>
+        <v>IKEv2</v>
       </c>
       <c r="C31" t="str">
-        <v>Group 14</v>
+        <v>IKEv2</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -2954,13 +2954,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Encryption Algorithm</v>
+        <v>Diffie-Hellman Group</v>
       </c>
       <c r="B32" t="str">
-        <v>AES256</v>
+        <v>Group 14</v>
       </c>
       <c r="C32" t="str">
-        <v>AES256</v>
+        <v>Group 14</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -3034,13 +3034,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Hashing Algorithm</v>
+        <v>Encryption Algorithm</v>
       </c>
       <c r="B33" t="str">
-        <v>SHA256</v>
+        <v>AES256</v>
       </c>
       <c r="C33" t="str">
-        <v>SHA256</v>
+        <v>AES256</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -3114,13 +3114,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Main or Aggressive Mode</v>
+        <v>Hashing Algorithm</v>
       </c>
       <c r="B34" t="str">
-        <v xml:space="preserve">Main </v>
+        <v>SHA256</v>
       </c>
       <c r="C34" t="str">
-        <v xml:space="preserve">Main </v>
+        <v>SHA256</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -3194,13 +3194,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Lifetime (for renegotiation)</v>
+        <v>Main or Aggressive Mode</v>
       </c>
       <c r="B35" t="str">
-        <v>86400s</v>
+        <v xml:space="preserve">Main </v>
       </c>
       <c r="C35" t="str">
-        <v>86400s</v>
+        <v xml:space="preserve">Main </v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -3274,13 +3274,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>IPSEC Phase 2 Parameters</v>
+        <v>Lifetime (for renegotiation)</v>
       </c>
       <c r="B36" t="str">
-        <v/>
+        <v>86400s</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>86400s</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -3354,13 +3354,13 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Encapsulation (ESP or AH)</v>
+        <v>IPSEC Phase 2 Parameters</v>
       </c>
       <c r="B37" t="str">
-        <v>ESP</v>
+        <v/>
       </c>
       <c r="C37" t="str">
-        <v>ESP</v>
+        <v/>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -3434,13 +3434,13 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Encryption Algorithm</v>
+        <v>Encapsulation (ESP or AH)</v>
       </c>
       <c r="B38" t="str">
-        <v>AES256</v>
+        <v>ESP</v>
       </c>
       <c r="C38" t="str">
-        <v>AES256</v>
+        <v>ESP</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -3514,13 +3514,13 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Authentication Algorithm</v>
+        <v>Encryption Algorithm</v>
       </c>
       <c r="B39" t="str">
-        <v>SHA256</v>
+        <v>AES256</v>
       </c>
       <c r="C39" t="str">
-        <v>SHA256</v>
+        <v>AES256</v>
       </c>
       <c r="D39" t="str">
         <v/>
@@ -3594,13 +3594,13 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Perfect Forward Secrecy</v>
+        <v>Authentication Algorithm</v>
       </c>
       <c r="B40" t="str">
-        <v>Disabled (preferred)</v>
+        <v>SHA256</v>
       </c>
       <c r="C40" t="str">
-        <v>Disabled (preferred)</v>
+        <v>SHA256</v>
       </c>
       <c r="D40" t="str">
         <v/>
@@ -3674,13 +3674,13 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Lifetime (for renegotiation)</v>
+        <v>Perfect Forward Secrecy</v>
       </c>
       <c r="B41" t="str">
-        <v>3600s</v>
+        <v>Disabled (preferred)</v>
       </c>
       <c r="C41" t="str">
-        <v>3600s</v>
+        <v>Disabled (preferred)</v>
       </c>
       <c r="D41" t="str">
         <v/>
@@ -3754,81 +3754,161 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
+        <v>Lifetime (for renegotiation)</v>
+      </c>
+      <c r="B42" t="str">
+        <v>3600s</v>
+      </c>
+      <c r="C42" t="str">
+        <v>3600s</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+      <c r="N42" t="str">
+        <v/>
+      </c>
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v/>
+      </c>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v/>
+      </c>
+      <c r="Z42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
         <v>Lifesize in KB (for renegotiation)</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B43" t="str">
         <v>N/A</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C43" t="str">
         <v>N/A</v>
       </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
-      <c r="E42" t="str">
-        <v/>
-      </c>
-      <c r="F42" t="str">
-        <v/>
-      </c>
-      <c r="G42" t="str">
-        <v/>
-      </c>
-      <c r="H42" t="str">
-        <v/>
-      </c>
-      <c r="I42" t="str">
-        <v/>
-      </c>
-      <c r="J42" t="str">
-        <v/>
-      </c>
-      <c r="K42" t="str">
-        <v/>
-      </c>
-      <c r="L42" t="str">
-        <v/>
-      </c>
-      <c r="M42" t="str">
-        <v/>
-      </c>
-      <c r="N42" t="str">
-        <v/>
-      </c>
-      <c r="O42" t="str">
-        <v/>
-      </c>
-      <c r="P42" t="str">
-        <v/>
-      </c>
-      <c r="Q42" t="str">
-        <v/>
-      </c>
-      <c r="R42" t="str">
-        <v/>
-      </c>
-      <c r="S42" t="str">
-        <v/>
-      </c>
-      <c r="T42" t="str">
-        <v/>
-      </c>
-      <c r="U42" t="str">
-        <v/>
-      </c>
-      <c r="V42" t="str">
-        <v/>
-      </c>
-      <c r="W42" t="str">
-        <v/>
-      </c>
-      <c r="X42" t="str">
-        <v/>
-      </c>
-      <c r="Y42" t="str">
-        <v/>
-      </c>
-      <c r="Z42" t="str">
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
+      <c r="M43" t="str">
+        <v/>
+      </c>
+      <c r="N43" t="str">
+        <v/>
+      </c>
+      <c r="O43" t="str">
+        <v/>
+      </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v/>
+      </c>
+      <c r="V43" t="str">
+        <v/>
+      </c>
+      <c r="W43" t="str">
+        <v/>
+      </c>
+      <c r="X43" t="str">
+        <v/>
+      </c>
+      <c r="Y43" t="str">
+        <v/>
+      </c>
+      <c r="Z43" t="str">
         <v/>
       </c>
     </row>
@@ -3837,7 +3917,7 @@
     <mergeCell ref="A3:C3"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z43"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>